<commit_message>
fix: update the function to calculate the protein structure based parameters
</commit_message>
<xml_diff>
--- a/data/proteomics/GEM_membrane_size_across_compartment_Rosemary_NH4_limitation_v2.xlsx
+++ b/data/proteomics/GEM_membrane_size_across_compartment_Rosemary_NH4_limitation_v2.xlsx
@@ -535,58 +535,58 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>130.0726989532351</v>
+        <v>130.185888895709</v>
       </c>
       <c r="D2" t="n">
-        <v>116.9214302731133</v>
+        <v>117.0220782874857</v>
       </c>
       <c r="E2" t="n">
-        <v>120.3235004292196</v>
+        <v>120.4422376030028</v>
       </c>
       <c r="F2" t="n">
-        <v>99.52368350625297</v>
+        <v>99.61704247581848</v>
       </c>
       <c r="G2" t="n">
-        <v>103.3938728541855</v>
+        <v>103.4945380789617</v>
       </c>
       <c r="H2" t="n">
-        <v>144.5979210992351</v>
+        <v>144.7475941534124</v>
       </c>
       <c r="I2" t="n">
-        <v>151.0223674873924</v>
+        <v>151.1898882276295</v>
       </c>
       <c r="J2" t="n">
-        <v>130.9169249271896</v>
+        <v>131.0524504264827</v>
       </c>
       <c r="K2" t="n">
-        <v>132.1745508285231</v>
+        <v>132.314185050436</v>
       </c>
       <c r="L2" t="n">
-        <v>141.5646080050194</v>
+        <v>141.7007061949118</v>
       </c>
       <c r="M2" t="n">
-        <v>141.7103155531431</v>
+        <v>141.8573585039967</v>
       </c>
       <c r="N2" t="n">
-        <v>146.9194487882636</v>
+        <v>147.0641318515164</v>
       </c>
       <c r="O2" t="n">
-        <v>253.0930600567281</v>
+        <v>253.3100363015902</v>
       </c>
       <c r="P2" t="n">
-        <v>256.6965097698234</v>
+        <v>256.909486960748</v>
       </c>
       <c r="Q2" t="n">
-        <v>237.165387305933</v>
+        <v>237.4043741250241</v>
       </c>
       <c r="R2" t="n">
-        <v>308.6285531691346</v>
+        <v>308.9041460065014</v>
       </c>
       <c r="S2" t="n">
-        <v>328.8540464220717</v>
+        <v>329.1749942806376</v>
       </c>
       <c r="T2" t="n">
-        <v>328.0688660071337</v>
+        <v>328.3331721584385</v>
       </c>
     </row>
     <row r="3">
@@ -666,55 +666,55 @@
         <v>0.0272198136760088</v>
       </c>
       <c r="D4" t="n">
-        <v>0.02489056226605527</v>
+        <v>0.04366081993521523</v>
       </c>
       <c r="E4" t="n">
-        <v>0.02662702620585459</v>
+        <v>0.05641644632609141</v>
       </c>
       <c r="F4" t="n">
-        <v>0.02903536435847641</v>
+        <v>0.06651237490589733</v>
       </c>
       <c r="G4" t="n">
-        <v>0.02896587406401615</v>
+        <v>0.06607867611736726</v>
       </c>
       <c r="H4" t="n">
         <v>0.05129209552171649</v>
       </c>
       <c r="I4" t="n">
-        <v>0.04936862485566569</v>
+        <v>0.09779130762590109</v>
       </c>
       <c r="J4" t="n">
-        <v>0.04140400008339046</v>
+        <v>0.08740228766209635</v>
       </c>
       <c r="K4" t="n">
-        <v>0.04176063012882297</v>
+        <v>0.06421105546883552</v>
       </c>
       <c r="L4" t="n">
         <v>0.04692922234797754</v>
       </c>
       <c r="M4" t="n">
-        <v>0.04596295754191636</v>
+        <v>0.1082174889011724</v>
       </c>
       <c r="N4" t="n">
-        <v>0.04908600942010151</v>
+        <v>0.1179683572956473</v>
       </c>
       <c r="O4" t="n">
-        <v>0.07177223093333977</v>
+        <v>0.130534302340421</v>
       </c>
       <c r="P4" t="n">
-        <v>0.06753680270978693</v>
+        <v>0.1577672110800275</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.06637260470137958</v>
+        <v>0.1421713453586584</v>
       </c>
       <c r="R4" t="n">
-        <v>0.07842620846674279</v>
+        <v>0.1574306842318353</v>
       </c>
       <c r="S4" t="n">
-        <v>0.07914331648172261</v>
+        <v>0.1348122328391508</v>
       </c>
       <c r="T4" t="n">
-        <v>0.08574005788635461</v>
+        <v>0.1943180086398622</v>
       </c>
     </row>
     <row r="5">
@@ -727,58 +727,58 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2.238725298216868</v>
+        <v>2.351236992604323</v>
       </c>
       <c r="D5" t="n">
-        <v>2.052120173093929</v>
+        <v>2.152327138416752</v>
       </c>
       <c r="E5" t="n">
-        <v>2.116253516134182</v>
+        <v>2.233419848226263</v>
       </c>
       <c r="F5" t="n">
-        <v>2.280349615218308</v>
+        <v>2.372663290849368</v>
       </c>
       <c r="G5" t="n">
-        <v>2.328769872138951</v>
+        <v>2.428511022928254</v>
       </c>
       <c r="H5" t="n">
-        <v>3.074399718692941</v>
+        <v>3.213952457026657</v>
       </c>
       <c r="I5" t="n">
-        <v>3.983039848826407</v>
+        <v>4.144868526854022</v>
       </c>
       <c r="J5" t="n">
-        <v>3.406499066154315</v>
+        <v>3.537406878517528</v>
       </c>
       <c r="K5" t="n">
-        <v>3.487038715952183</v>
+        <v>3.621649943418223</v>
       </c>
       <c r="L5" t="n">
-        <v>4.279518573887892</v>
+        <v>4.41394834200265</v>
       </c>
       <c r="M5" t="n">
-        <v>4.245488033519699</v>
+        <v>4.387840860978494</v>
       </c>
       <c r="N5" t="n">
-        <v>4.082295944692448</v>
+        <v>4.223515026967146</v>
       </c>
       <c r="O5" t="n">
-        <v>7.439911290550959</v>
+        <v>7.648622197085769</v>
       </c>
       <c r="P5" t="n">
-        <v>7.842436411434861</v>
+        <v>8.046936177142971</v>
       </c>
       <c r="Q5" t="n">
-        <v>6.845949560147099</v>
+        <v>7.078029064078855</v>
       </c>
       <c r="R5" t="n">
-        <v>8.396705105982198</v>
+        <v>8.665164758794436</v>
       </c>
       <c r="S5" t="n">
-        <v>8.774994165223525</v>
+        <v>9.081459010771381</v>
       </c>
       <c r="T5" t="n">
-        <v>8.828105556590573</v>
+        <v>9.082828840579783</v>
       </c>
     </row>
     <row r="6">
@@ -791,55 +791,55 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>50.51276258625929</v>
+        <v>50.51309380439933</v>
       </c>
       <c r="D6" t="n">
-        <v>44.7936759259341</v>
+        <v>44.79396217026801</v>
       </c>
       <c r="E6" t="n">
-        <v>48.08699966554709</v>
+        <v>48.08723109054397</v>
       </c>
       <c r="F6" t="n">
-        <v>42.61370275661428</v>
+        <v>42.61394200212533</v>
       </c>
       <c r="G6" t="n">
-        <v>43.73049365614996</v>
+        <v>43.73049365614995</v>
       </c>
       <c r="H6" t="n">
-        <v>54.05776074980028</v>
+        <v>54.05809549860032</v>
       </c>
       <c r="I6" t="n">
-        <v>62.58691763155492</v>
+        <v>62.58747027359786</v>
       </c>
       <c r="J6" t="n">
         <v>56.21018133262449</v>
       </c>
       <c r="K6" t="n">
-        <v>54.35402758367957</v>
+        <v>54.35451352412515</v>
       </c>
       <c r="L6" t="n">
-        <v>55.99596895982207</v>
+        <v>55.99659947941499</v>
       </c>
       <c r="M6" t="n">
-        <v>58.10883959975494</v>
+        <v>58.10949645382041</v>
       </c>
       <c r="N6" t="n">
         <v>60.38101094863509</v>
       </c>
       <c r="O6" t="n">
-        <v>103.1197015542868</v>
+        <v>103.1214230843597</v>
       </c>
       <c r="P6" t="n">
-        <v>103.647078410773</v>
+        <v>103.6492743617218</v>
       </c>
       <c r="Q6" t="n">
-        <v>99.33969742097769</v>
+        <v>99.34137066442511</v>
       </c>
       <c r="R6" t="n">
-        <v>132.7499160496762</v>
+        <v>132.7525162145216</v>
       </c>
       <c r="S6" t="n">
-        <v>145.3702322657038</v>
+        <v>145.3724720915574</v>
       </c>
       <c r="T6" t="n">
         <v>133.0159078288335</v>
@@ -855,58 +855,58 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>109.481136395385</v>
+        <v>109.5490026500852</v>
       </c>
       <c r="D7" t="n">
-        <v>98.47213170560326</v>
+        <v>98.47410106421256</v>
       </c>
       <c r="E7" t="n">
-        <v>101.205397696529</v>
+        <v>101.2720414146269</v>
       </c>
       <c r="F7" t="n">
-        <v>86.50101562215232</v>
+        <v>86.50325454022</v>
       </c>
       <c r="G7" t="n">
-        <v>91.44204727850797</v>
+        <v>91.51103647261841</v>
       </c>
       <c r="H7" t="n">
-        <v>123.8678198006946</v>
+        <v>123.9237297959135</v>
       </c>
       <c r="I7" t="n">
-        <v>128.9237020809534</v>
+        <v>128.9277101649658</v>
       </c>
       <c r="J7" t="n">
-        <v>109.3937721695879</v>
+        <v>109.4692428034937</v>
       </c>
       <c r="K7" t="n">
-        <v>112.2505811096255</v>
+        <v>112.2538174242108</v>
       </c>
       <c r="L7" t="n">
-        <v>129.8708527429453</v>
+        <v>129.9385103365995</v>
       </c>
       <c r="M7" t="n">
-        <v>126.4263385982958</v>
+        <v>126.4875045058653</v>
       </c>
       <c r="N7" t="n">
-        <v>127.6990290676654</v>
+        <v>127.7861840707352</v>
       </c>
       <c r="O7" t="n">
-        <v>238.2808268468505</v>
+        <v>238.2887487165489</v>
       </c>
       <c r="P7" t="n">
-        <v>240.9633166649585</v>
+        <v>241.0321507055305</v>
       </c>
       <c r="Q7" t="n">
-        <v>234.9722672312897</v>
+        <v>234.9805683548713</v>
       </c>
       <c r="R7" t="n">
-        <v>307.7522241224202</v>
+        <v>307.8400051304656</v>
       </c>
       <c r="S7" t="n">
-        <v>317.0729327883574</v>
+        <v>317.0846071196093</v>
       </c>
       <c r="T7" t="n">
-        <v>322.2775522829435</v>
+        <v>322.4120428738858</v>
       </c>
     </row>
     <row r="8">
@@ -919,58 +919,58 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>68.60053818949073</v>
+        <v>68.6663226954384</v>
       </c>
       <c r="D8" t="n">
-        <v>58.44996247188371</v>
+        <v>58.44996247188369</v>
       </c>
       <c r="E8" t="n">
-        <v>59.82991790625834</v>
+        <v>59.89606118876956</v>
       </c>
       <c r="F8" t="n">
-        <v>52.4858308424676</v>
+        <v>52.48643672488533</v>
       </c>
       <c r="G8" t="n">
-        <v>53.06223050771943</v>
+        <v>53.13028345492638</v>
       </c>
       <c r="H8" t="n">
-        <v>85.13876486776061</v>
+        <v>85.19186813013481</v>
       </c>
       <c r="I8" t="n">
-        <v>83.007610587958</v>
+        <v>83.00843541097679</v>
       </c>
       <c r="J8" t="n">
-        <v>72.55338526663546</v>
+        <v>72.62662367473717</v>
       </c>
       <c r="K8" t="n">
         <v>70.06081154651851</v>
       </c>
       <c r="L8" t="n">
-        <v>69.46731953857511</v>
+        <v>69.53203636150501</v>
       </c>
       <c r="M8" t="n">
-        <v>72.77619715707961</v>
+        <v>72.83656589728338</v>
       </c>
       <c r="N8" t="n">
-        <v>73.7900812662871</v>
+        <v>73.87521256810082</v>
       </c>
       <c r="O8" t="n">
-        <v>139.2328532706716</v>
+        <v>139.2328532706717</v>
       </c>
       <c r="P8" t="n">
-        <v>140.1196042175076</v>
+        <v>140.1861248772562</v>
       </c>
       <c r="Q8" t="n">
-        <v>134.2429830308271</v>
+        <v>134.2442084848554</v>
       </c>
       <c r="R8" t="n">
-        <v>187.9653435738584</v>
+        <v>188.050107213832</v>
       </c>
       <c r="S8" t="n">
-        <v>210.3285886791469</v>
+        <v>210.3298159495379</v>
       </c>
       <c r="T8" t="n">
-        <v>195.3679672133835</v>
+        <v>195.4943758804535</v>
       </c>
     </row>
     <row r="9">
@@ -1139,58 +1139,58 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>4.738923597209006</v>
+        <v>4.850893885468254</v>
       </c>
       <c r="D12" t="n">
-        <v>4.23498920087149</v>
+        <v>4.335196166194311</v>
       </c>
       <c r="E12" t="n">
-        <v>4.428262155521404</v>
+        <v>4.544736276748555</v>
       </c>
       <c r="F12" t="n">
-        <v>4.027572573097203</v>
+        <v>4.119280366310551</v>
       </c>
       <c r="G12" t="n">
-        <v>4.556311590409567</v>
+        <v>4.655466747107662</v>
       </c>
       <c r="H12" t="n">
-        <v>4.848900986641629</v>
+        <v>4.988003101902447</v>
       </c>
       <c r="I12" t="n">
-        <v>7.327147270621963</v>
+        <v>7.488151125630784</v>
       </c>
       <c r="J12" t="n">
-        <v>6.28498115308448</v>
+        <v>6.415232821592061</v>
       </c>
       <c r="K12" t="n">
-        <v>6.348672755815691</v>
+        <v>6.483283983281729</v>
       </c>
       <c r="L12" t="n">
-        <v>7.599898254714787</v>
+        <v>7.733345439428096</v>
       </c>
       <c r="M12" t="n">
-        <v>6.965421488432029</v>
+        <v>7.106973747428484</v>
       </c>
       <c r="N12" t="n">
-        <v>7.555535769920832</v>
+        <v>7.695795353395592</v>
       </c>
       <c r="O12" t="n">
-        <v>10.90988567740378</v>
+        <v>11.11859658393859</v>
       </c>
       <c r="P12" t="n">
-        <v>11.25476168545357</v>
+        <v>11.45797500558583</v>
       </c>
       <c r="Q12" t="n">
-        <v>11.11899303846982</v>
+        <v>11.34984708837334</v>
       </c>
       <c r="R12" t="n">
-        <v>12.34009632253372</v>
+        <v>12.60726703364597</v>
       </c>
       <c r="S12" t="n">
-        <v>12.79303396384315</v>
+        <v>13.098271539</v>
       </c>
       <c r="T12" t="n">
-        <v>13.4161210549753</v>
+        <v>13.66945050134808</v>
       </c>
     </row>
     <row r="13">
@@ -1267,58 +1267,58 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2.169795425898629</v>
+        <v>2.281765714157876</v>
       </c>
       <c r="D14" t="n">
-        <v>1.992195358035002</v>
+        <v>2.092402323357824</v>
       </c>
       <c r="E14" t="n">
-        <v>2.025825710841883</v>
+        <v>2.142299832069034</v>
       </c>
       <c r="F14" t="n">
-        <v>1.517922464558379</v>
+        <v>1.609630257771726</v>
       </c>
       <c r="G14" t="n">
-        <v>1.709970535772992</v>
+        <v>1.809125692471087</v>
       </c>
       <c r="H14" t="n">
-        <v>2.184533872164692</v>
+        <v>2.32363598742551</v>
       </c>
       <c r="I14" t="n">
-        <v>2.697334330383459</v>
+        <v>2.85833818539228</v>
       </c>
       <c r="J14" t="n">
-        <v>2.221269681441805</v>
+        <v>2.351521349949385</v>
       </c>
       <c r="K14" t="n">
-        <v>2.322213994702705</v>
+        <v>2.456825222168745</v>
       </c>
       <c r="L14" t="n">
-        <v>2.701028224268714</v>
+        <v>2.834475408982022</v>
       </c>
       <c r="M14" t="n">
-        <v>2.665137793018963</v>
+        <v>2.806690052015413</v>
       </c>
       <c r="N14" t="n">
-        <v>2.691869859972497</v>
+        <v>2.832129443447258</v>
       </c>
       <c r="O14" t="n">
-        <v>4.083671022724741</v>
+        <v>4.29238192925955</v>
       </c>
       <c r="P14" t="n">
-        <v>4.189869498723906</v>
+        <v>4.393082818856169</v>
       </c>
       <c r="Q14" t="n">
-        <v>3.590790258791595</v>
+        <v>3.821644308695122</v>
       </c>
       <c r="R14" t="n">
-        <v>4.371834318405045</v>
+        <v>4.639005029517292</v>
       </c>
       <c r="S14" t="n">
-        <v>4.126525463301304</v>
+        <v>4.43176303845816</v>
       </c>
       <c r="T14" t="n">
-        <v>4.780333560879079</v>
+        <v>5.033663007251857</v>
       </c>
     </row>
     <row r="15">
@@ -1358,7 +1358,7 @@
         <v>0.3073627492125124</v>
       </c>
       <c r="L15" t="n">
-        <v>0.3142456517905975</v>
+        <v>0.3142456517905976</v>
       </c>
       <c r="M15" t="n">
         <v>0.3030887227167997</v>
@@ -1370,7 +1370,7 @@
         <v>0.3503143855739134</v>
       </c>
       <c r="P15" t="n">
-        <v>0.3813340949270076</v>
+        <v>0.3813340949270077</v>
       </c>
       <c r="Q15" t="n">
         <v>0.2952611910425086</v>
@@ -1398,55 +1398,55 @@
         <v>0.6111194048790487</v>
       </c>
       <c r="D16" t="n">
-        <v>0.538175068547412</v>
+        <v>0.556945326216572</v>
       </c>
       <c r="E16" t="n">
-        <v>0.537014027859859</v>
+        <v>0.5668034479800957</v>
       </c>
       <c r="F16" t="n">
-        <v>0.6069588623455986</v>
+        <v>0.6444358728930197</v>
       </c>
       <c r="G16" t="n">
-        <v>0.6323231907613502</v>
+        <v>0.6694359928147012</v>
       </c>
       <c r="H16" t="n">
         <v>0.5860366713004249</v>
       </c>
       <c r="I16" t="n">
-        <v>1.000233953840431</v>
+        <v>1.048656636610666</v>
       </c>
       <c r="J16" t="n">
-        <v>0.8654924063403601</v>
+        <v>0.911490693919066</v>
       </c>
       <c r="K16" t="n">
-        <v>0.8813889215800005</v>
+        <v>0.903839346920013</v>
       </c>
       <c r="L16" t="n">
         <v>1.123334261644729</v>
       </c>
       <c r="M16" t="n">
-        <v>1.099947265090878</v>
+        <v>1.162201796450134</v>
       </c>
       <c r="N16" t="n">
-        <v>1.133134632319001</v>
+        <v>1.202016980194546</v>
       </c>
       <c r="O16" t="n">
-        <v>1.833725619295137</v>
+        <v>1.892487690702218</v>
       </c>
       <c r="P16" t="n">
-        <v>1.757339226825613</v>
+        <v>1.847569635195854</v>
       </c>
       <c r="Q16" t="n">
-        <v>1.726662229066378</v>
+        <v>1.802460969723656</v>
       </c>
       <c r="R16" t="n">
-        <v>2.228312275442786</v>
+        <v>2.307316751207878</v>
       </c>
       <c r="S16" t="n">
-        <v>2.283138337865499</v>
+        <v>2.338807254222927</v>
       </c>
       <c r="T16" t="n">
-        <v>2.275314738347464</v>
+        <v>2.383892689100972</v>
       </c>
     </row>
     <row r="17">
@@ -1459,58 +1459,58 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1.229567540877847</v>
+        <v>1.230108947006054</v>
       </c>
       <c r="D17" t="n">
         <v>1.059703931683007</v>
       </c>
       <c r="E17" t="n">
-        <v>1.094503681328116</v>
+        <v>1.095195892193046</v>
       </c>
       <c r="F17" t="n">
-        <v>1.106597661788095</v>
+        <v>1.107203544205809</v>
       </c>
       <c r="G17" t="n">
-        <v>1.328027804037642</v>
+        <v>1.328613798128851</v>
       </c>
       <c r="H17" t="n">
-        <v>0.9772885072978267</v>
+        <v>0.9777391303707247</v>
       </c>
       <c r="I17" t="n">
-        <v>2.021059557954703</v>
+        <v>2.021884380973499</v>
       </c>
       <c r="J17" t="n">
-        <v>1.612088848787301</v>
+        <v>1.612744992642934</v>
       </c>
       <c r="K17" t="n">
-        <v>1.802061070842347</v>
+        <v>1.802061070842346</v>
       </c>
       <c r="L17" t="n">
-        <v>2.02897335813683</v>
+        <v>2.029955941538279</v>
       </c>
       <c r="M17" t="n">
-        <v>1.713393744973942</v>
+        <v>1.714194313436286</v>
       </c>
       <c r="N17" t="n">
-        <v>2.074872554441035</v>
+        <v>2.075832053240971</v>
       </c>
       <c r="O17" t="n">
-        <v>2.426525689703754</v>
+        <v>2.426525689703753</v>
       </c>
       <c r="P17" t="n">
-        <v>2.278409795077</v>
+        <v>2.279696240652843</v>
       </c>
       <c r="Q17" t="n">
-        <v>2.273695179350302</v>
+        <v>2.274920633378532</v>
       </c>
       <c r="R17" t="n">
-        <v>2.016599159800308</v>
+        <v>2.0178881015003</v>
       </c>
       <c r="S17" t="n">
-        <v>1.909060975188666</v>
+        <v>1.910288245579665</v>
       </c>
       <c r="T17" t="n">
-        <v>2.435347193704999</v>
+        <v>2.436741031321429</v>
       </c>
     </row>
     <row r="18">
@@ -1523,58 +1523,58 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.1126146122572646</v>
+        <v>0.2245849005165119</v>
       </c>
       <c r="D18" t="n">
-        <v>0.09632798171521752</v>
+        <v>0.1965349470380401</v>
       </c>
       <c r="E18" t="n">
-        <v>0.1072983605607587</v>
+        <v>0.2237724817879102</v>
       </c>
       <c r="F18" t="n">
-        <v>0.1236594864354606</v>
+        <v>0.2153672796488073</v>
       </c>
       <c r="G18" t="n">
-        <v>0.1275238897503927</v>
+        <v>0.2266790464484872</v>
       </c>
       <c r="H18" t="n">
-        <v>0.1076620756951689</v>
+        <v>0.2467641909559867</v>
       </c>
       <c r="I18" t="n">
-        <v>0.1965163447959492</v>
+        <v>0.3575201998047692</v>
       </c>
       <c r="J18" t="n">
-        <v>0.1831535459921027</v>
+        <v>0.3134052144996831</v>
       </c>
       <c r="K18" t="n">
-        <v>0.1809843422464489</v>
+        <v>0.3155955697124894</v>
       </c>
       <c r="L18" t="n">
-        <v>0.2427345039115813</v>
+        <v>0.3761816886248899</v>
       </c>
       <c r="M18" t="n">
-        <v>0.2288241874143706</v>
+        <v>0.3703764464108215</v>
       </c>
       <c r="N18" t="n">
-        <v>0.2438305154535806</v>
+        <v>0.3840900989283421</v>
       </c>
       <c r="O18" t="n">
-        <v>0.3649385801923063</v>
+        <v>0.5736494867271166</v>
       </c>
       <c r="P18" t="n">
-        <v>0.368923314442267</v>
+        <v>0.5721366345745315</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.4358093151941961</v>
+        <v>0.666663365097721</v>
       </c>
       <c r="R18" t="n">
-        <v>0.4958570493529209</v>
+        <v>0.7630277604651661</v>
       </c>
       <c r="S18" t="n">
-        <v>0.5470191587392292</v>
+        <v>0.8522567338960854</v>
       </c>
       <c r="T18" t="n">
-        <v>0.5403310262840273</v>
+        <v>0.7936604726568065</v>
       </c>
     </row>
     <row r="19">
@@ -1587,58 +1587,58 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.2571029336940218</v>
+        <v>0.3690732219532691</v>
       </c>
       <c r="D19" t="n">
-        <v>0.2186937713239582</v>
+        <v>0.3189007366467809</v>
       </c>
       <c r="E19" t="n">
-        <v>0.240051150770949</v>
+        <v>0.3565252719981005</v>
       </c>
       <c r="F19" t="n">
-        <v>0.2791048277958277</v>
+        <v>0.3708126210091744</v>
       </c>
       <c r="G19" t="n">
-        <v>0.2832348608207266</v>
+        <v>0.3823900175188211</v>
       </c>
       <c r="H19" t="n">
-        <v>0.2384338792703746</v>
+        <v>0.3775359945311925</v>
       </c>
       <c r="I19" t="n">
-        <v>0.4161535040342491</v>
+        <v>0.577157359043069</v>
       </c>
       <c r="J19" t="n">
-        <v>0.3823445630949775</v>
+        <v>0.512596231602558</v>
       </c>
       <c r="K19" t="n">
-        <v>0.3794159831861054</v>
+        <v>0.5140272106521458</v>
       </c>
       <c r="L19" t="n">
-        <v>0.4862143778377321</v>
+        <v>0.6196615625510407</v>
       </c>
       <c r="M19" t="n">
-        <v>0.4621431303214487</v>
+        <v>0.6036953893178995</v>
       </c>
       <c r="N19" t="n">
-        <v>0.4947046021969869</v>
+        <v>0.6349641856717484</v>
       </c>
       <c r="O19" t="n">
-        <v>0.6922714551644044</v>
+        <v>0.9009823616992146</v>
       </c>
       <c r="P19" t="n">
-        <v>0.6920456608177616</v>
+        <v>0.8952589809500261</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.7808573385829937</v>
+        <v>1.011711388486519</v>
       </c>
       <c r="R19" t="n">
-        <v>0.9042014283621072</v>
+        <v>1.171372139474352</v>
       </c>
       <c r="S19" t="n">
-        <v>0.9382311923880319</v>
+        <v>1.243468767544888</v>
       </c>
       <c r="T19" t="n">
-        <v>0.967519420471869</v>
+        <v>1.220848866844648</v>
       </c>
     </row>
     <row r="20">
@@ -1651,58 +1651,58 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2.267437385257348</v>
+        <v>2.379407673516595</v>
       </c>
       <c r="D20" t="n">
-        <v>1.937159369289156</v>
+        <v>2.037366334611978</v>
       </c>
       <c r="E20" t="n">
-        <v>2.269756411742463</v>
+        <v>2.386230532969615</v>
       </c>
       <c r="F20" t="n">
-        <v>2.157916083549817</v>
+        <v>2.249623876763164</v>
       </c>
       <c r="G20" t="n">
-        <v>2.340984998843914</v>
+        <v>2.440140155542008</v>
       </c>
       <c r="H20" t="n">
-        <v>2.957767392688841</v>
+        <v>3.096869507949659</v>
       </c>
       <c r="I20" t="n">
-        <v>3.262691557968103</v>
+        <v>3.423695412976923</v>
       </c>
       <c r="J20" t="n">
-        <v>2.795785074499069</v>
+        <v>2.92603674300665</v>
       </c>
       <c r="K20" t="n">
-        <v>2.914384360309089</v>
+        <v>3.04899558777513</v>
       </c>
       <c r="L20" t="n">
-        <v>3.934544359040945</v>
+        <v>4.067991543754253</v>
       </c>
       <c r="M20" t="n">
-        <v>4.072945795899341</v>
+        <v>4.214498054895792</v>
       </c>
       <c r="N20" t="n">
-        <v>3.327964269896077</v>
+        <v>3.468223853370838</v>
       </c>
       <c r="O20" t="n">
-        <v>8.635660362699472</v>
+        <v>8.844371269234282</v>
       </c>
       <c r="P20" t="n">
-        <v>8.435047854988484</v>
+        <v>8.638261175120748</v>
       </c>
       <c r="Q20" t="n">
-        <v>8.311611758022984</v>
+        <v>8.54246580792651</v>
       </c>
       <c r="R20" t="n">
-        <v>10.55938806415959</v>
+        <v>10.82655877527184</v>
       </c>
       <c r="S20" t="n">
-        <v>9.102577162166419</v>
+        <v>9.407814737323275</v>
       </c>
       <c r="T20" t="n">
-        <v>11.21452526056344</v>
+        <v>11.46785470693622</v>
       </c>
     </row>
     <row r="21">
@@ -1807,13 +1807,13 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>20.21381550307476</v>
+        <v>20.21381550307477</v>
       </c>
       <c r="D23" t="n">
         <v>16.10736033483598</v>
       </c>
       <c r="E23" t="n">
-        <v>13.89610281862554</v>
+        <v>13.89610281862555</v>
       </c>
       <c r="F23" t="n">
         <v>12.43672842661202</v>
@@ -1828,7 +1828,7 @@
         <v>25.19160963354679</v>
       </c>
       <c r="J23" t="n">
-        <v>21.14765070885778</v>
+        <v>21.14765070885777</v>
       </c>
       <c r="K23" t="n">
         <v>19.91920690220537</v>
@@ -1843,7 +1843,7 @@
         <v>18.13950646199186</v>
       </c>
       <c r="O23" t="n">
-        <v>40.6814596707035</v>
+        <v>40.68145967070351</v>
       </c>
       <c r="P23" t="n">
         <v>42.24091808220334</v>
@@ -1858,7 +1858,7 @@
         <v>73.63419542367332</v>
       </c>
       <c r="T23" t="n">
-        <v>60.58080551424214</v>
+        <v>60.58080551424215</v>
       </c>
     </row>
     <row r="24">
@@ -1963,58 +1963,58 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>0.1126146122572646</v>
+        <v>0.2245849005165119</v>
       </c>
       <c r="D26" t="n">
-        <v>0.09632798171521752</v>
+        <v>0.1965349470380401</v>
       </c>
       <c r="E26" t="n">
-        <v>0.1072983605607587</v>
+        <v>0.2237724817879102</v>
       </c>
       <c r="F26" t="n">
-        <v>0.1236594864354606</v>
+        <v>0.2153672796488073</v>
       </c>
       <c r="G26" t="n">
-        <v>0.1275238897503927</v>
+        <v>0.2266790464484872</v>
       </c>
       <c r="H26" t="n">
-        <v>0.1076620756951689</v>
+        <v>0.2467641909559867</v>
       </c>
       <c r="I26" t="n">
-        <v>0.1965163447959492</v>
+        <v>0.3575201998047692</v>
       </c>
       <c r="J26" t="n">
-        <v>0.1831535459921027</v>
+        <v>0.3134052144996831</v>
       </c>
       <c r="K26" t="n">
-        <v>0.1809843422464489</v>
+        <v>0.3155955697124894</v>
       </c>
       <c r="L26" t="n">
-        <v>0.2427345039115813</v>
+        <v>0.3761816886248899</v>
       </c>
       <c r="M26" t="n">
-        <v>0.2288241874143706</v>
+        <v>0.3703764464108215</v>
       </c>
       <c r="N26" t="n">
-        <v>0.2438305154535806</v>
+        <v>0.3840900989283421</v>
       </c>
       <c r="O26" t="n">
-        <v>0.3649385801923063</v>
+        <v>0.5736494867271166</v>
       </c>
       <c r="P26" t="n">
-        <v>0.368923314442267</v>
+        <v>0.5721366345745315</v>
       </c>
       <c r="Q26" t="n">
-        <v>0.4358093151941961</v>
+        <v>0.666663365097721</v>
       </c>
       <c r="R26" t="n">
-        <v>0.4958570493529209</v>
+        <v>0.7630277604651661</v>
       </c>
       <c r="S26" t="n">
-        <v>0.5470191587392292</v>
+        <v>0.8522567338960854</v>
       </c>
       <c r="T26" t="n">
-        <v>0.5403310262840273</v>
+        <v>0.7936604726568065</v>
       </c>
     </row>
     <row r="27">
@@ -2155,58 +2155,58 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>5.548689543161403</v>
+        <v>5.661201237548856</v>
       </c>
       <c r="D29" t="n">
-        <v>5.305166938308171</v>
+        <v>5.40537390363099</v>
       </c>
       <c r="E29" t="n">
-        <v>5.170384852950083</v>
+        <v>5.287551185042163</v>
       </c>
       <c r="F29" t="n">
-        <v>5.250265134301198</v>
+        <v>5.342578809932258</v>
       </c>
       <c r="G29" t="n">
-        <v>6.203601703211835</v>
+        <v>6.303342854001138</v>
       </c>
       <c r="H29" t="n">
-        <v>4.430861369393726</v>
+        <v>4.570414107727442</v>
       </c>
       <c r="I29" t="n">
-        <v>6.162891527424826</v>
+        <v>6.324720205452441</v>
       </c>
       <c r="J29" t="n">
-        <v>5.432625522573871</v>
+        <v>5.563533334937084</v>
       </c>
       <c r="K29" t="n">
-        <v>6.31212356915486</v>
+        <v>6.446734796620898</v>
       </c>
       <c r="L29" t="n">
-        <v>7.154674163302055</v>
+        <v>7.289103931416813</v>
       </c>
       <c r="M29" t="n">
-        <v>6.73517479519161</v>
+        <v>6.877527622650404</v>
       </c>
       <c r="N29" t="n">
-        <v>7.148317760667157</v>
+        <v>7.289536842941856</v>
       </c>
       <c r="O29" t="n">
-        <v>10.85024594451962</v>
+        <v>11.05895685105442</v>
       </c>
       <c r="P29" t="n">
-        <v>11.18624791273888</v>
+        <v>11.39074767844699</v>
       </c>
       <c r="Q29" t="n">
-        <v>11.09806938133603</v>
+        <v>11.33014888526779</v>
       </c>
       <c r="R29" t="n">
-        <v>12.68122569707982</v>
+        <v>12.94968534989206</v>
       </c>
       <c r="S29" t="n">
-        <v>10.70040346311429</v>
+        <v>11.00686830866215</v>
       </c>
       <c r="T29" t="n">
-        <v>13.3367981640121</v>
+        <v>13.5915214480013</v>
       </c>
     </row>
     <row r="30">
@@ -2275,40 +2275,40 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>6.369819075466666</v>
+        <v>6.369819075466668</v>
       </c>
       <c r="D32" t="n">
-        <v>5.850748981355576</v>
+        <v>5.850748981355575</v>
       </c>
       <c r="E32" t="n">
         <v>6.781505547568267</v>
       </c>
       <c r="F32" t="n">
-        <v>6.167765128579926</v>
+        <v>6.167765128579927</v>
       </c>
       <c r="G32" t="n">
-        <v>6.864766003431789</v>
+        <v>6.864766003431788</v>
       </c>
       <c r="H32" t="n">
         <v>8.051716962354725</v>
       </c>
       <c r="I32" t="n">
-        <v>8.80529868979424</v>
+        <v>8.805298689794242</v>
       </c>
       <c r="J32" t="n">
-        <v>7.586225551758502</v>
+        <v>7.586225551758501</v>
       </c>
       <c r="K32" t="n">
         <v>7.666000324686706</v>
       </c>
       <c r="L32" t="n">
-        <v>9.197283115375267</v>
+        <v>9.197283115375269</v>
       </c>
       <c r="M32" t="n">
-        <v>9.449359405226897</v>
+        <v>9.449359405226899</v>
       </c>
       <c r="N32" t="n">
-        <v>9.485563149902012</v>
+        <v>9.485563149902015</v>
       </c>
       <c r="O32" t="n">
         <v>18.20347314068038</v>
@@ -2320,7 +2320,7 @@
         <v>17.39288402707375</v>
       </c>
       <c r="R32" t="n">
-        <v>23.03228464590263</v>
+        <v>23.03228464590262</v>
       </c>
       <c r="S32" t="n">
         <v>26.34395377305301</v>
@@ -2354,7 +2354,7 @@
         <v>14.17896001957998</v>
       </c>
       <c r="H33" t="n">
-        <v>14.87483032348907</v>
+        <v>14.87483032348906</v>
       </c>
       <c r="I33" t="n">
         <v>18.35483524025688</v>
@@ -2402,24 +2402,60 @@
           <t>incipient cellular bud site</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
-      <c r="Q34" t="inlineStr"/>
-      <c r="R34" t="inlineStr"/>
-      <c r="S34" t="inlineStr"/>
-      <c r="T34" t="inlineStr"/>
+      <c r="C34" t="n">
+        <v>0.1119702882592473</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0.1002069653228226</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0.1164741212271515</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.09170779321334668</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0.09915515669809449</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0.1391021152608179</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0.1610038550088199</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0.1302516685075804</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0.1346112274660405</v>
+      </c>
+      <c r="L34" t="n">
+        <v>0.1334471847133085</v>
+      </c>
+      <c r="M34" t="n">
+        <v>0.1415522589964509</v>
+      </c>
+      <c r="N34" t="n">
+        <v>0.1402595834747614</v>
+      </c>
+      <c r="O34" t="n">
+        <v>0.2087109065348103</v>
+      </c>
+      <c r="P34" t="n">
+        <v>0.2032133201322644</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>0.2308540499035249</v>
+      </c>
+      <c r="R34" t="n">
+        <v>0.2671707111122452</v>
+      </c>
+      <c r="S34" t="n">
+        <v>0.3052375751568562</v>
+      </c>
+      <c r="T34" t="n">
+        <v>0.2533294463727793</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
@@ -2498,7 +2534,7 @@
         <v>0.02512281254728653</v>
       </c>
       <c r="D36" t="n">
-        <v>0.02109415125900425</v>
+        <v>0.02109415125900424</v>
       </c>
       <c r="E36" t="n">
         <v>0.02795738015486242</v>
@@ -2510,10 +2546,10 @@
         <v>0.02571722150694136</v>
       </c>
       <c r="H36" t="n">
-        <v>0.02957535177005469</v>
+        <v>0.02957535177005468</v>
       </c>
       <c r="I36" t="n">
-        <v>0.04042148854811859</v>
+        <v>0.04042148854811858</v>
       </c>
       <c r="J36" t="n">
         <v>0.0364785110445672</v>
@@ -2522,7 +2558,7 @@
         <v>0.03462618139385066</v>
       </c>
       <c r="L36" t="n">
-        <v>0.04605253589001634</v>
+        <v>0.04605253589001632</v>
       </c>
       <c r="M36" t="n">
         <v>0.04305525586734567</v>
@@ -2534,19 +2570,19 @@
         <v>0.07291822142404468</v>
       </c>
       <c r="P36" t="n">
-        <v>0.07185003788358515</v>
+        <v>0.07185003788358517</v>
       </c>
       <c r="Q36" t="n">
         <v>0.07997571785696014</v>
       </c>
       <c r="R36" t="n">
-        <v>0.08653750130980177</v>
+        <v>0.08653750130980176</v>
       </c>
       <c r="S36" t="n">
         <v>0.1042630837611117</v>
       </c>
       <c r="T36" t="n">
-        <v>0.0972840866284841</v>
+        <v>0.09728408662848412</v>
       </c>
     </row>
     <row r="37">
@@ -2559,58 +2595,58 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>4.957712433596175</v>
+        <v>4.954091835329042</v>
       </c>
       <c r="D37" t="n">
-        <v>4.045146515813659</v>
+        <v>4.04174645603131</v>
       </c>
       <c r="E37" t="n">
-        <v>4.476141374880352</v>
+        <v>4.472707711143337</v>
       </c>
       <c r="F37" t="n">
-        <v>4.001615123060162</v>
+        <v>3.99848684575145</v>
       </c>
       <c r="G37" t="n">
-        <v>4.216976225606836</v>
+        <v>4.213793830106287</v>
       </c>
       <c r="H37" t="n">
-        <v>6.686370422865934</v>
+        <v>6.684013322262593</v>
       </c>
       <c r="I37" t="n">
-        <v>7.52456451473719</v>
+        <v>7.520494014947201</v>
       </c>
       <c r="J37" t="n">
-        <v>6.679034905004984</v>
+        <v>6.675657119358279</v>
       </c>
       <c r="K37" t="n">
-        <v>6.825492492192534</v>
+        <v>6.821741278273781</v>
       </c>
       <c r="L37" t="n">
-        <v>7.728639992124931</v>
+        <v>7.724259498624487</v>
       </c>
       <c r="M37" t="n">
-        <v>7.446051947270332</v>
+        <v>7.441940427566628</v>
       </c>
       <c r="N37" t="n">
-        <v>7.335115905488599</v>
+        <v>7.330695466660988</v>
       </c>
       <c r="O37" t="n">
-        <v>11.14028375139434</v>
+        <v>11.13389647506639</v>
       </c>
       <c r="P37" t="n">
-        <v>11.74352863407096</v>
+        <v>11.73731083125584</v>
       </c>
       <c r="Q37" t="n">
-        <v>10.08645123505949</v>
+        <v>10.0808567738169</v>
       </c>
       <c r="R37" t="n">
-        <v>12.47149337231779</v>
+        <v>12.46495092781593</v>
       </c>
       <c r="S37" t="n">
-        <v>11.25065451447623</v>
+        <v>11.24440141122662</v>
       </c>
       <c r="T37" t="n">
-        <v>13.25265277853751</v>
+        <v>13.24514063707295</v>
       </c>
     </row>
     <row r="38">
@@ -2787,13 +2823,13 @@
         <v>0.08298847573781691</v>
       </c>
       <c r="K43" t="n">
-        <v>0.09272478125410369</v>
+        <v>0.09272478125410367</v>
       </c>
       <c r="L43" t="n">
         <v>0.1004443194993656</v>
       </c>
       <c r="M43" t="n">
-        <v>0.09584902381599143</v>
+        <v>0.09584902381599145</v>
       </c>
       <c r="N43" t="n">
         <v>0.1062861448824326</v>
@@ -2802,7 +2838,7 @@
         <v>0.1436390671273954</v>
       </c>
       <c r="P43" t="n">
-        <v>0.1481715626329129</v>
+        <v>0.148171562632913</v>
       </c>
       <c r="Q43" t="n">
         <v>0.1353133931242047</v>
@@ -2827,58 +2863,58 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>0.06600157660404339</v>
+        <v>0.1779718648632908</v>
       </c>
       <c r="D44" t="n">
-        <v>0.0604475276652293</v>
+        <v>0.1606544929880518</v>
       </c>
       <c r="E44" t="n">
-        <v>0.05810469077231518</v>
+        <v>0.1745788119994667</v>
       </c>
       <c r="F44" t="n">
-        <v>0.05874100651006221</v>
+        <v>0.1504487997234089</v>
       </c>
       <c r="G44" t="n">
-        <v>0.06106687147556656</v>
+        <v>0.160222028173661</v>
       </c>
       <c r="H44" t="n">
-        <v>0.06152719659175709</v>
+        <v>0.200629311852575</v>
       </c>
       <c r="I44" t="n">
-        <v>0.09290792561777643</v>
+        <v>0.2539117806265963</v>
       </c>
       <c r="J44" t="n">
-        <v>0.08013555698526413</v>
+        <v>0.2103872254928446</v>
       </c>
       <c r="K44" t="n">
-        <v>0.08398334853967611</v>
+        <v>0.2185945760057166</v>
       </c>
       <c r="L44" t="n">
-        <v>0.1071689688171818</v>
+        <v>0.2406161535304903</v>
       </c>
       <c r="M44" t="n">
-        <v>0.09917220823663248</v>
+        <v>0.2407244672330834</v>
       </c>
       <c r="N44" t="n">
-        <v>0.1030923658498047</v>
+        <v>0.2433519493245661</v>
       </c>
       <c r="O44" t="n">
-        <v>0.1736930069625836</v>
+        <v>0.3824039134973939</v>
       </c>
       <c r="P44" t="n">
-        <v>0.1818555100731047</v>
+        <v>0.3850688302053691</v>
       </c>
       <c r="Q44" t="n">
-        <v>0.1836656955034491</v>
+        <v>0.414519745406974</v>
       </c>
       <c r="R44" t="n">
-        <v>0.2218328319453423</v>
+        <v>0.4890035430575874</v>
       </c>
       <c r="S44" t="n">
-        <v>0.2239434411459314</v>
+        <v>0.5291810163027876</v>
       </c>
       <c r="T44" t="n">
-        <v>0.236935706675566</v>
+        <v>0.4902651530483453</v>
       </c>
     </row>
     <row r="45">
@@ -3011,7 +3047,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>0.2096368489793872</v>
+        <v>0.2096368489793871</v>
       </c>
       <c r="D48" t="n">
         <v>0.1751279356662966</v>
@@ -3041,7 +3077,7 @@
         <v>0.1264651296135138</v>
       </c>
       <c r="M48" t="n">
-        <v>0.1176583254549038</v>
+        <v>0.1176583254549039</v>
       </c>
       <c r="N48" t="n">
         <v>0.1154676745908176</v>
@@ -3254,7 +3290,7 @@
         <v>14.27250130284631</v>
       </c>
       <c r="D54" t="n">
-        <v>13.00862877227459</v>
+        <v>13.0086287722746</v>
       </c>
       <c r="E54" t="n">
         <v>12.34143222796795</v>
@@ -3263,7 +3299,7 @@
         <v>9.038679439805646</v>
       </c>
       <c r="G54" t="n">
-        <v>10.06595495762201</v>
+        <v>10.06595495762202</v>
       </c>
       <c r="H54" t="n">
         <v>13.08374531184747</v>
@@ -3284,25 +3320,25 @@
         <v>10.65759194358525</v>
       </c>
       <c r="N54" t="n">
-        <v>10.98952476152553</v>
+        <v>10.98952476152554</v>
       </c>
       <c r="O54" t="n">
         <v>25.51841529890842</v>
       </c>
       <c r="P54" t="n">
-        <v>24.58058627471989</v>
+        <v>24.5805862747199</v>
       </c>
       <c r="Q54" t="n">
         <v>25.20444519008123</v>
       </c>
       <c r="R54" t="n">
-        <v>39.35162918324443</v>
+        <v>39.35162918324444</v>
       </c>
       <c r="S54" t="n">
-        <v>40.97005555104434</v>
+        <v>40.97005555104435</v>
       </c>
       <c r="T54" t="n">
-        <v>40.61412986910048</v>
+        <v>40.61412986910049</v>
       </c>
     </row>
     <row r="55">
@@ -3315,16 +3351,16 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>0.8634459177934325</v>
+        <v>0.8634459177934323</v>
       </c>
       <c r="D55" t="n">
-        <v>0.7616490965814351</v>
+        <v>0.761649096581435</v>
       </c>
       <c r="E55" t="n">
-        <v>0.7402465886180823</v>
+        <v>0.7402465886180825</v>
       </c>
       <c r="F55" t="n">
-        <v>0.8599641289725479</v>
+        <v>0.859964128972548</v>
       </c>
       <c r="G55" t="n">
         <v>0.8943006512810988</v>
@@ -3363,7 +3399,7 @@
         <v>2.148778566039036</v>
       </c>
       <c r="S55" t="n">
-        <v>2.231500312307248</v>
+        <v>2.231500312307247</v>
       </c>
       <c r="T55" t="n">
         <v>2.251259558112976</v>
@@ -3379,13 +3415,13 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>8.382644208685269</v>
+        <v>8.382644208685267</v>
       </c>
       <c r="D56" t="n">
-        <v>7.425252216044982</v>
+        <v>7.425252216044983</v>
       </c>
       <c r="E56" t="n">
-        <v>7.761106999758656</v>
+        <v>7.761106999758654</v>
       </c>
       <c r="F56" t="n">
         <v>8.911688697361464</v>
@@ -3394,7 +3430,7 @@
         <v>9.332502739699621</v>
       </c>
       <c r="H56" t="n">
-        <v>9.256634189370867</v>
+        <v>9.256634189370866</v>
       </c>
       <c r="I56" t="n">
         <v>15.16379703254192</v>
@@ -3427,10 +3463,10 @@
         <v>24.85611584618271</v>
       </c>
       <c r="S56" t="n">
-        <v>28.2229337735774</v>
+        <v>28.22293377357739</v>
       </c>
       <c r="T56" t="n">
-        <v>30.74311531963916</v>
+        <v>30.74311531963915</v>
       </c>
     </row>
     <row r="57">
@@ -3499,58 +3535,58 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>0.01252383292031001</v>
+        <v>0.07776693273974329</v>
       </c>
       <c r="D59" t="n">
         <v>0.01083557259272475</v>
       </c>
       <c r="E59" t="n">
-        <v>0.01217039614947553</v>
+        <v>0.07762146779576454</v>
       </c>
       <c r="F59" t="n">
         <v>0.01255215855169689</v>
       </c>
       <c r="G59" t="n">
-        <v>0.01131713126110345</v>
+        <v>0.07878408437682935</v>
       </c>
       <c r="H59" t="n">
-        <v>0.01236531659064726</v>
+        <v>0.0650179558919558</v>
       </c>
       <c r="I59" t="n">
         <v>0.01873246162226155</v>
       </c>
       <c r="J59" t="n">
-        <v>0.01689990100766683</v>
+        <v>0.0894821652537361</v>
       </c>
       <c r="K59" t="n">
         <v>0.01483145590637942</v>
       </c>
       <c r="L59" t="n">
-        <v>0.01779792406928145</v>
+        <v>0.08153216359768409</v>
       </c>
       <c r="M59" t="n">
-        <v>0.02220495293615586</v>
+        <v>0.08177312467760729</v>
       </c>
       <c r="N59" t="n">
-        <v>0.02006545814690759</v>
+        <v>0.1042372611606703</v>
       </c>
       <c r="O59" t="n">
         <v>0.03932848523836977</v>
       </c>
       <c r="P59" t="n">
-        <v>0.05084786842871986</v>
+        <v>0.1160820826015571</v>
       </c>
       <c r="Q59" t="n">
         <v>0.02311780307832095</v>
       </c>
       <c r="R59" t="n">
-        <v>0.05842236964378996</v>
+        <v>0.1418970679173507</v>
       </c>
       <c r="S59" t="n">
         <v>0.05510175087519414</v>
       </c>
       <c r="T59" t="n">
-        <v>0.05492132560231396</v>
+        <v>0.1799361550558748</v>
       </c>
     </row>
     <row r="60">
@@ -3584,16 +3620,16 @@
         <v>7.239607556833382</v>
       </c>
       <c r="J60" t="n">
-        <v>6.387024526805232</v>
+        <v>6.387024526805233</v>
       </c>
       <c r="K60" t="n">
         <v>6.375002716506289</v>
       </c>
       <c r="L60" t="n">
-        <v>7.118125329716436</v>
+        <v>7.118125329716437</v>
       </c>
       <c r="M60" t="n">
-        <v>6.833038671207972</v>
+        <v>6.833038671207974</v>
       </c>
       <c r="N60" t="n">
         <v>7.554527735779766</v>
@@ -3602,7 +3638,7 @@
         <v>10.46621010601849</v>
       </c>
       <c r="P60" t="n">
-        <v>10.22337146679512</v>
+        <v>10.22337146679511</v>
       </c>
       <c r="Q60" t="n">
         <v>10.88084801284613</v>
@@ -3627,58 +3663,58 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>0.0004200716842741366</v>
+        <v>0.002193335092265955</v>
       </c>
       <c r="D61" t="n">
-        <v>0.0004711109912461015</v>
+        <v>0.001431547520797278</v>
       </c>
       <c r="E61" t="n">
-        <v>0.0004328352695592723</v>
+        <v>0.002086267589216431</v>
       </c>
       <c r="F61" t="n">
-        <v>0.0004034412660674956</v>
+        <v>0.001853433979065134</v>
       </c>
       <c r="G61" t="n">
-        <v>0.000440745699846909</v>
+        <v>0.001936177788664004</v>
       </c>
       <c r="H61" t="n">
-        <v>0.0003102971770383663</v>
+        <v>0.001699119062412189</v>
       </c>
       <c r="I61" t="n">
-        <v>0.0004315481388105973</v>
+        <v>0.002255135552122728</v>
       </c>
       <c r="J61" t="n">
-        <v>0.0003552971511748769</v>
+        <v>0.001967529421998297</v>
       </c>
       <c r="K61" t="n">
-        <v>0.0004808438911643926</v>
+        <v>0.001262931542377566</v>
       </c>
       <c r="L61" t="n">
-        <v>0.0004795185230478943</v>
+        <v>0.00230259183749603</v>
       </c>
       <c r="M61" t="n">
-        <v>0.000384662405962462</v>
+        <v>0.002126112630816487</v>
       </c>
       <c r="N61" t="n">
-        <v>0.0005166075017750821</v>
+        <v>0.00257633259430136</v>
       </c>
       <c r="O61" t="n">
-        <v>0.0006196854464968447</v>
+        <v>0.001623437560093304</v>
       </c>
       <c r="P61" t="n">
-        <v>0.0006132462211372567</v>
+        <v>0.003303567247437566</v>
       </c>
       <c r="Q61" t="n">
-        <v>0.000762432965410681</v>
+        <v>0.002888185590172635</v>
       </c>
       <c r="R61" t="n">
-        <v>0.0006633431441274073</v>
+        <v>0.003658429770290395</v>
       </c>
       <c r="S61" t="n">
-        <v>0.0006788248983928218</v>
+        <v>0.002853834629641257</v>
       </c>
       <c r="T61" t="n">
-        <v>0.0006945735506067595</v>
+        <v>0.003474990712004004</v>
       </c>
     </row>
     <row r="62">
@@ -3690,24 +3726,60 @@
           <t>vacuole-isolation membrane contact site</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr"/>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
-      <c r="M62" t="inlineStr"/>
-      <c r="N62" t="inlineStr"/>
-      <c r="O62" t="inlineStr"/>
-      <c r="P62" t="inlineStr"/>
-      <c r="Q62" t="inlineStr"/>
-      <c r="R62" t="inlineStr"/>
-      <c r="S62" t="inlineStr"/>
-      <c r="T62" t="inlineStr"/>
+      <c r="C62" t="n">
+        <v>0.0652430998194333</v>
+      </c>
+      <c r="D62" t="n">
+        <v>0</v>
+      </c>
+      <c r="E62" t="n">
+        <v>0.06545107164628901</v>
+      </c>
+      <c r="F62" t="n">
+        <v>0</v>
+      </c>
+      <c r="G62" t="n">
+        <v>0.06746695311572593</v>
+      </c>
+      <c r="H62" t="n">
+        <v>0.05265263930130854</v>
+      </c>
+      <c r="I62" t="n">
+        <v>0</v>
+      </c>
+      <c r="J62" t="n">
+        <v>0.07258226424606927</v>
+      </c>
+      <c r="K62" t="n">
+        <v>0</v>
+      </c>
+      <c r="L62" t="n">
+        <v>0.06373423952840264</v>
+      </c>
+      <c r="M62" t="n">
+        <v>0.05956817174145145</v>
+      </c>
+      <c r="N62" t="n">
+        <v>0.08417180301376272</v>
+      </c>
+      <c r="O62" t="n">
+        <v>0</v>
+      </c>
+      <c r="P62" t="n">
+        <v>0.06523421417283728</v>
+      </c>
+      <c r="Q62" t="n">
+        <v>0</v>
+      </c>
+      <c r="R62" t="n">
+        <v>0.08347469827356074</v>
+      </c>
+      <c r="S62" t="n">
+        <v>0</v>
+      </c>
+      <c r="T62" t="n">
+        <v>0.1250148294535608</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
@@ -3728,7 +3800,7 @@
         <v>3.642964943835539</v>
       </c>
       <c r="F63" t="n">
-        <v>2.927147888791542</v>
+        <v>2.927147888791543</v>
       </c>
       <c r="G63" t="n">
         <v>3.551649495801326</v>
@@ -3737,7 +3809,7 @@
         <v>4.718196288977957</v>
       </c>
       <c r="I63" t="n">
-        <v>4.301913159242302</v>
+        <v>4.301913159242303</v>
       </c>
       <c r="J63" t="n">
         <v>4.149946445067632</v>
@@ -3746,31 +3818,31 @@
         <v>3.914138564424056</v>
       </c>
       <c r="L63" t="n">
-        <v>3.657154975435667</v>
+        <v>3.657154975435668</v>
       </c>
       <c r="M63" t="n">
-        <v>3.946878782076351</v>
+        <v>3.94687878207635</v>
       </c>
       <c r="N63" t="n">
-        <v>4.717068892437197</v>
+        <v>4.717068892437196</v>
       </c>
       <c r="O63" t="n">
         <v>4.650873907000145</v>
       </c>
       <c r="P63" t="n">
-        <v>4.799371575464302</v>
+        <v>4.799371575464303</v>
       </c>
       <c r="Q63" t="n">
         <v>4.039804227423646</v>
       </c>
       <c r="R63" t="n">
-        <v>5.836515091961093</v>
+        <v>5.836515091961092</v>
       </c>
       <c r="S63" t="n">
         <v>6.074457666597573</v>
       </c>
       <c r="T63" t="n">
-        <v>4.881479087232996</v>
+        <v>4.881479087232997</v>
       </c>
     </row>
     <row r="64">
@@ -3847,19 +3919,19 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>11.9074618109064</v>
+        <v>11.90746181090639</v>
       </c>
       <c r="D65" t="n">
-        <v>11.52060061506453</v>
+        <v>11.52060061506452</v>
       </c>
       <c r="E65" t="n">
-        <v>11.51691963386305</v>
+        <v>11.51691963386304</v>
       </c>
       <c r="F65" t="n">
         <v>5.867269113836714</v>
       </c>
       <c r="G65" t="n">
-        <v>6.39002804743836</v>
+        <v>6.390028047438359</v>
       </c>
       <c r="H65" t="n">
         <v>10.08607042001789</v>
@@ -3871,7 +3943,7 @@
         <v>8.145972420471868</v>
       </c>
       <c r="K65" t="n">
-        <v>8.578483037925174</v>
+        <v>8.578483037925173</v>
       </c>
       <c r="L65" t="n">
         <v>10.09140573733985</v>
@@ -3880,13 +3952,13 @@
         <v>9.583308265868229</v>
       </c>
       <c r="N65" t="n">
-        <v>9.981487091601243</v>
+        <v>9.981487091601245</v>
       </c>
       <c r="O65" t="n">
         <v>16.10657100003728</v>
       </c>
       <c r="P65" t="n">
-        <v>16.93590522342729</v>
+        <v>16.93590522342728</v>
       </c>
       <c r="Q65" t="n">
         <v>13.80696413706823</v>
@@ -3898,7 +3970,7 @@
         <v>16.06207161434048</v>
       </c>
       <c r="T65" t="n">
-        <v>18.29349836406923</v>
+        <v>18.29349836406924</v>
       </c>
     </row>
     <row r="66">
@@ -3914,13 +3986,13 @@
         <v>0.02829992684498785</v>
       </c>
       <c r="D66" t="n">
-        <v>0.02597922612503274</v>
+        <v>0.02597922612503273</v>
       </c>
       <c r="E66" t="n">
-        <v>0.02565221034783777</v>
+        <v>0.02565221034783778</v>
       </c>
       <c r="F66" t="n">
-        <v>0.02243888527989689</v>
+        <v>0.02243888527989688</v>
       </c>
       <c r="G66" t="n">
         <v>0.02491567204304139</v>
@@ -3944,19 +4016,19 @@
         <v>0.0336258573049811</v>
       </c>
       <c r="N66" t="n">
-        <v>0.03346400001627009</v>
+        <v>0.0334640000162701</v>
       </c>
       <c r="O66" t="n">
         <v>0.04894201425993187</v>
       </c>
       <c r="P66" t="n">
-        <v>0.05066747350584213</v>
+        <v>0.05066747350584212</v>
       </c>
       <c r="Q66" t="n">
         <v>0.0542664307198819</v>
       </c>
       <c r="R66" t="n">
-        <v>0.05560065340874169</v>
+        <v>0.0556006534087417</v>
       </c>
       <c r="S66" t="n">
         <v>0.07434132587662813</v>
@@ -4123,7 +4195,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>3.137226718909273</v>
+        <v>3.137226718909272</v>
       </c>
       <c r="D71" t="n">
         <v>2.654863805858439</v>
@@ -4168,7 +4240,7 @@
         <v>8.601536626665625</v>
       </c>
       <c r="R71" t="n">
-        <v>10.45315437339849</v>
+        <v>10.45315437339848</v>
       </c>
       <c r="S71" t="n">
         <v>10.40139199543582</v>
@@ -4199,7 +4271,7 @@
         <v>1.502198500212197</v>
       </c>
       <c r="G72" t="n">
-        <v>1.475601813658419</v>
+        <v>1.475601813658418</v>
       </c>
       <c r="H72" t="n">
         <v>1.62018703407056</v>
@@ -4208,10 +4280,10 @@
         <v>2.37124719532207</v>
       </c>
       <c r="J72" t="n">
-        <v>1.953750323763862</v>
+        <v>1.953750323763863</v>
       </c>
       <c r="K72" t="n">
-        <v>2.111841838724905</v>
+        <v>2.111841838724904</v>
       </c>
       <c r="L72" t="n">
         <v>2.570043846652989</v>
@@ -4229,7 +4301,7 @@
         <v>5.204499656144019</v>
       </c>
       <c r="Q72" t="n">
-        <v>4.310597322480882</v>
+        <v>4.310597322480883</v>
       </c>
       <c r="R72" t="n">
         <v>6.175678152968787</v>
@@ -4238,7 +4310,7 @@
         <v>5.214370953027129</v>
       </c>
       <c r="T72" t="n">
-        <v>6.721981905591028</v>
+        <v>6.721981905591029</v>
       </c>
     </row>
     <row r="73">
@@ -4251,58 +4323,58 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>0.7736224160055515</v>
+        <v>0.8855927042647986</v>
       </c>
       <c r="D73" t="n">
-        <v>0.7141237787468692</v>
+        <v>0.8143307440696916</v>
       </c>
       <c r="E73" t="n">
-        <v>0.713630515401611</v>
+        <v>0.8301046366287622</v>
       </c>
       <c r="F73" t="n">
-        <v>0.6653852861608159</v>
+        <v>0.7570930793741626</v>
       </c>
       <c r="G73" t="n">
-        <v>0.6880785870023967</v>
+        <v>0.7872337437004913</v>
       </c>
       <c r="H73" t="n">
-        <v>0.9836128395407708</v>
+        <v>1.122714954801588</v>
       </c>
       <c r="I73" t="n">
-        <v>1.128615043200032</v>
+        <v>1.289618898208852</v>
       </c>
       <c r="J73" t="n">
-        <v>0.9082917177734917</v>
+        <v>1.038543386281072</v>
       </c>
       <c r="K73" t="n">
-        <v>0.9950179224205422</v>
+        <v>1.129629149886583</v>
       </c>
       <c r="L73" t="n">
-        <v>1.17825185672419</v>
+        <v>1.311699041437499</v>
       </c>
       <c r="M73" t="n">
-        <v>1.121759199473814</v>
+        <v>1.263311458470265</v>
       </c>
       <c r="N73" t="n">
-        <v>1.090721871105778</v>
+        <v>1.230981454580539</v>
       </c>
       <c r="O73" t="n">
-        <v>1.598700317240893</v>
+        <v>1.807411223775703</v>
       </c>
       <c r="P73" t="n">
-        <v>1.766789999357711</v>
+        <v>1.970003319489975</v>
       </c>
       <c r="Q73" t="n">
-        <v>1.518623243308965</v>
+        <v>1.749477293212489</v>
       </c>
       <c r="R73" t="n">
-        <v>1.832312794178893</v>
+        <v>2.099483505291138</v>
       </c>
       <c r="S73" t="n">
-        <v>1.801557290779029</v>
+        <v>2.106794865935885</v>
       </c>
       <c r="T73" t="n">
-        <v>1.94256724061818</v>
+        <v>2.195896686990959</v>
       </c>
     </row>
     <row r="74">
@@ -4357,7 +4429,7 @@
         <v>0.4260118188494135</v>
       </c>
       <c r="Q74" t="n">
-        <v>0.3370471796433114</v>
+        <v>0.3370471796433113</v>
       </c>
       <c r="R74" t="n">
         <v>0.4747375477914674</v>
@@ -4646,24 +4718,60 @@
           <t>mitochondrial ribosome</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr"/>
-      <c r="D82" t="inlineStr"/>
-      <c r="E82" t="inlineStr"/>
-      <c r="F82" t="inlineStr"/>
-      <c r="G82" t="inlineStr"/>
-      <c r="H82" t="inlineStr"/>
-      <c r="I82" t="inlineStr"/>
-      <c r="J82" t="inlineStr"/>
-      <c r="K82" t="inlineStr"/>
-      <c r="L82" t="inlineStr"/>
-      <c r="M82" t="inlineStr"/>
-      <c r="N82" t="inlineStr"/>
-      <c r="O82" t="inlineStr"/>
-      <c r="P82" t="inlineStr"/>
-      <c r="Q82" t="inlineStr"/>
-      <c r="R82" t="inlineStr"/>
-      <c r="S82" t="inlineStr"/>
-      <c r="T82" t="inlineStr"/>
+      <c r="C82" t="n">
+        <v>0.00700450988282006</v>
+      </c>
+      <c r="D82" t="n">
+        <v>0.005702365754814037</v>
+      </c>
+      <c r="E82" t="n">
+        <v>0.007353944538080957</v>
+      </c>
+      <c r="F82" t="n">
+        <v>0.006816313609888727</v>
+      </c>
+      <c r="G82" t="n">
+        <v>0.006746759373897219</v>
+      </c>
+      <c r="H82" t="n">
+        <v>0.01475948985483937</v>
+      </c>
+      <c r="I82" t="n">
+        <v>0.01423507280567535</v>
+      </c>
+      <c r="J82" t="n">
+        <v>0.0115521245536134</v>
+      </c>
+      <c r="K82" t="n">
+        <v>0.0118972177844137</v>
+      </c>
+      <c r="L82" t="n">
+        <v>0.01153417394177573</v>
+      </c>
+      <c r="M82" t="n">
+        <v>0.01355660442747202</v>
+      </c>
+      <c r="N82" t="n">
+        <v>0.01286873432911663</v>
+      </c>
+      <c r="O82" t="n">
+        <v>0.02272425227755953</v>
+      </c>
+      <c r="P82" t="n">
+        <v>0.02431598769644333</v>
+      </c>
+      <c r="Q82" t="n">
+        <v>0.02185318710777564</v>
+      </c>
+      <c r="R82" t="n">
+        <v>0.02420732255629593</v>
+      </c>
+      <c r="S82" t="n">
+        <v>0.03024414150696486</v>
+      </c>
+      <c r="T82" t="n">
+        <v>0.02853571901375441</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="n">
@@ -4714,7 +4822,7 @@
         <v>5.75971813586441</v>
       </c>
       <c r="P83" t="n">
-        <v>6.161777009505934</v>
+        <v>6.161777009505935</v>
       </c>
       <c r="Q83" t="n">
         <v>5.259860609033285</v>
@@ -4754,13 +4862,13 @@
         <v>0.25709283860528</v>
       </c>
       <c r="H84" t="n">
-        <v>0.4351067700628225</v>
+        <v>0.4351067700628226</v>
       </c>
       <c r="I84" t="n">
         <v>0.4738288426401983</v>
       </c>
       <c r="J84" t="n">
-        <v>0.4291113378539253</v>
+        <v>0.4291113378539252</v>
       </c>
       <c r="K84" t="n">
         <v>0.4010874693766239</v>
@@ -5455,58 +5563,58 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>0.006047955163956524</v>
+        <v>0.002427356896821579</v>
       </c>
       <c r="D98" t="n">
-        <v>0.005647486795140778</v>
+        <v>0.002247427012791538</v>
       </c>
       <c r="E98" t="n">
-        <v>0.005796668037807824</v>
+        <v>0.002363004300792461</v>
       </c>
       <c r="F98" t="n">
-        <v>0.005179921025963303</v>
+        <v>0.002051643717250338</v>
       </c>
       <c r="G98" t="n">
-        <v>0.005318147867209628</v>
+        <v>0.002135752366659827</v>
       </c>
       <c r="H98" t="n">
-        <v>0.004546198261499723</v>
+        <v>0.002189097658156555</v>
       </c>
       <c r="I98" t="n">
-        <v>0.007299738780819161</v>
+        <v>0.003229238990830715</v>
       </c>
       <c r="J98" t="n">
-        <v>0.006166584868786684</v>
+        <v>0.002788799222080805</v>
       </c>
       <c r="K98" t="n">
-        <v>0.006570575249887428</v>
+        <v>0.002819361331132825</v>
       </c>
       <c r="L98" t="n">
-        <v>0.008276690657250247</v>
+        <v>0.003896197156806449</v>
       </c>
       <c r="M98" t="n">
-        <v>0.007963835902763795</v>
+        <v>0.003852316199059645</v>
       </c>
       <c r="N98" t="n">
-        <v>0.008207689871349663</v>
+        <v>0.003787251043738655</v>
       </c>
       <c r="O98" t="n">
-        <v>0.01281502144796933</v>
+        <v>0.006427745120023594</v>
       </c>
       <c r="P98" t="n">
-        <v>0.0128169853606882</v>
+        <v>0.006599182545575085</v>
       </c>
       <c r="Q98" t="n">
-        <v>0.01228238687375639</v>
+        <v>0.00668792563116529</v>
       </c>
       <c r="R98" t="n">
-        <v>0.0132030344336212</v>
+        <v>0.006660589931768211</v>
       </c>
       <c r="S98" t="n">
-        <v>0.01425441973754769</v>
+        <v>0.008001316487927708</v>
       </c>
       <c r="T98" t="n">
-        <v>0.01627487440768774</v>
+        <v>0.008762732943132444</v>
       </c>
     </row>
     <row r="99">
@@ -5694,24 +5802,60 @@
           <t>vacuolar membrane</t>
         </is>
       </c>
-      <c r="C104" t="inlineStr"/>
-      <c r="D104" t="inlineStr"/>
-      <c r="E104" t="inlineStr"/>
-      <c r="F104" t="inlineStr"/>
-      <c r="G104" t="inlineStr"/>
-      <c r="H104" t="inlineStr"/>
-      <c r="I104" t="inlineStr"/>
-      <c r="J104" t="inlineStr"/>
-      <c r="K104" t="inlineStr"/>
-      <c r="L104" t="inlineStr"/>
-      <c r="M104" t="inlineStr"/>
-      <c r="N104" t="inlineStr"/>
-      <c r="O104" t="inlineStr"/>
-      <c r="P104" t="inlineStr"/>
-      <c r="Q104" t="inlineStr"/>
-      <c r="R104" t="inlineStr"/>
-      <c r="S104" t="inlineStr"/>
-      <c r="T104" t="inlineStr"/>
+      <c r="C104" t="n">
+        <v>0.001231857279784671</v>
+      </c>
+      <c r="D104" t="n">
+        <v>0.0009604365295511766</v>
+      </c>
+      <c r="E104" t="n">
+        <v>0.0009612214547272143</v>
+      </c>
+      <c r="F104" t="n">
+        <v>0.0008441102952835138</v>
+      </c>
+      <c r="G104" t="n">
+        <v>0.0009094379976087865</v>
+      </c>
+      <c r="H104" t="n">
+        <v>0.0009381988124757009</v>
+      </c>
+      <c r="I104" t="n">
+        <v>0.0009987643945161527</v>
+      </c>
+      <c r="J104" t="n">
+        <v>0.0009560884151898711</v>
+      </c>
+      <c r="K104" t="n">
+        <v>0.0007820876512131737</v>
+      </c>
+      <c r="L104" t="n">
+        <v>0.0008404899129994298</v>
+      </c>
+      <c r="M104" t="n">
+        <v>0.0009408817625106286</v>
+      </c>
+      <c r="N104" t="n">
+        <v>0.00110022629259032</v>
+      </c>
+      <c r="O104" t="n">
+        <v>0.001003752113596459</v>
+      </c>
+      <c r="P104" t="n">
+        <v>0.00140387545045705</v>
+      </c>
+      <c r="Q104" t="n">
+        <v>0.0009002985965307416</v>
+      </c>
+      <c r="R104" t="n">
+        <v>0.001706144926170493</v>
+      </c>
+      <c r="S104" t="n">
+        <v>0.0009477393402494513</v>
+      </c>
+      <c r="T104" t="n">
+        <v>0.001386579544966635</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="1" t="n">
@@ -5932,10 +6076,10 @@
         <v>0.1881385140493518</v>
       </c>
       <c r="N110" t="n">
-        <v>0.1932500887452609</v>
+        <v>0.193250088745261</v>
       </c>
       <c r="O110" t="n">
-        <v>0.3133784444673172</v>
+        <v>0.3133784444673173</v>
       </c>
       <c r="P110" t="n">
         <v>0.3451279815988144</v>
@@ -6786,24 +6930,60 @@
           <t>phagophore</t>
         </is>
       </c>
-      <c r="C134" t="inlineStr"/>
-      <c r="D134" t="inlineStr"/>
-      <c r="E134" t="inlineStr"/>
-      <c r="F134" t="inlineStr"/>
-      <c r="G134" t="inlineStr"/>
-      <c r="H134" t="inlineStr"/>
-      <c r="I134" t="inlineStr"/>
-      <c r="J134" t="inlineStr"/>
-      <c r="K134" t="inlineStr"/>
-      <c r="L134" t="inlineStr"/>
-      <c r="M134" t="inlineStr"/>
-      <c r="N134" t="inlineStr"/>
-      <c r="O134" t="inlineStr"/>
-      <c r="P134" t="inlineStr"/>
-      <c r="Q134" t="inlineStr"/>
-      <c r="R134" t="inlineStr"/>
-      <c r="S134" t="inlineStr"/>
-      <c r="T134" t="inlineStr"/>
+      <c r="C134" t="n">
+        <v>0.0005414061282071475</v>
+      </c>
+      <c r="D134" t="n">
+        <v>0</v>
+      </c>
+      <c r="E134" t="n">
+        <v>0.0006922108649299445</v>
+      </c>
+      <c r="F134" t="n">
+        <v>0.0006058824177141243</v>
+      </c>
+      <c r="G134" t="n">
+        <v>0.0005859940912083083</v>
+      </c>
+      <c r="H134" t="n">
+        <v>0.000450623072898122</v>
+      </c>
+      <c r="I134" t="n">
+        <v>0.0008248230187959775</v>
+      </c>
+      <c r="J134" t="n">
+        <v>0.0006561438556335488</v>
+      </c>
+      <c r="K134" t="n">
+        <v>0</v>
+      </c>
+      <c r="L134" t="n">
+        <v>0.0009825834014487061</v>
+      </c>
+      <c r="M134" t="n">
+        <v>0.0008005684623433966</v>
+      </c>
+      <c r="N134" t="n">
+        <v>0.0009594987999359572</v>
+      </c>
+      <c r="O134" t="n">
+        <v>0</v>
+      </c>
+      <c r="P134" t="n">
+        <v>0.00128644557584326</v>
+      </c>
+      <c r="Q134" t="n">
+        <v>0.001225454028231212</v>
+      </c>
+      <c r="R134" t="n">
+        <v>0.001288941699992494</v>
+      </c>
+      <c r="S134" t="n">
+        <v>0.001227270390998983</v>
+      </c>
+      <c r="T134" t="n">
+        <v>0.00139383761643061</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="n">

</xml_diff>